<commit_message>
Enhance FormFiller class with error handling and logging for major and minor head selections
- Added detailed logging for major and minor head Excel values.
- Implemented error handling to raise ValueErrors when major or minor head sections are not found.
- Ensured dropdown options are verified after selection, with logging for successful matches.
- Improved visibility checks for major and minor head sections to ensure they are displayed before interaction.
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Automation\egram_bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DF4BCD-043E-452F-AD73-084B1A4AB9CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A741823A-05DE-4C25-9AD9-95FCC88A0145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,12 +20,15 @@
     <sheet name="Beneficiaries" sheetId="5" r:id="rId5"/>
     <sheet name="Asset" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Activities!$A$1:$AG$2</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="87">
   <si>
     <t>Activity_Key</t>
   </si>
@@ -273,41 +276,26 @@
     <t>Save and Forward</t>
   </si>
   <si>
-    <t>Theme 3 - Child Friendly Village</t>
-  </si>
-  <si>
-    <t>Education</t>
-  </si>
-  <si>
-    <t>Women and child development</t>
-  </si>
-  <si>
-    <t>ACT-0070</t>
-  </si>
-  <si>
-    <t>Child Participation, Leadership Strengthening &amp; Facilitation</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0081</t>
-  </si>
-  <si>
-    <t>Institutional Strengthening &amp; Convergence on child related issues</t>
-  </si>
-  <si>
-    <t>National Health Mission (NHM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Whether the activity is for Elementary/Primary Education</t>
+    <t>Theme 1 - Poverty Free and Enhanced Livelihoods Village</t>
+  </si>
+  <si>
+    <t>Poverty allevation programme</t>
+  </si>
+  <si>
+    <t>ACT-0028</t>
+  </si>
+  <si>
+    <t>Organise career counselling camps to promote self-employment opportunities at the GP level</t>
+  </si>
+  <si>
+    <t>Matsaya Yojna - Center Scheme</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -333,12 +321,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF231917"/>
-      <name val="Courier New"/>
-      <family val="3"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -354,32 +336,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFBFF"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -397,7 +364,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG3"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -737,7 +704,7 @@
     <col min="33" max="33" width="13.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -838,15 +805,15 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>85</v>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>84</v>
       </c>
       <c r="B2" t="s">
         <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D2" t="s">
         <v>83</v>
@@ -855,7 +822,7 @@
         <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I2" t="s">
         <v>76</v>
@@ -866,9 +833,6 @@
       <c r="K2" t="s">
         <v>77</v>
       </c>
-      <c r="M2" s="4" t="s">
-        <v>91</v>
-      </c>
       <c r="N2" t="s">
         <v>78</v>
       </c>
@@ -888,107 +852,30 @@
         <v>79</v>
       </c>
       <c r="T2">
+        <v>7</v>
+      </c>
+      <c r="U2">
+        <v>3</v>
+      </c>
+      <c r="V2">
+        <v>5</v>
+      </c>
+      <c r="W2">
         <v>9</v>
       </c>
-      <c r="U2">
-        <v>7</v>
-      </c>
-      <c r="V2">
-        <v>8</v>
-      </c>
-      <c r="W2">
-        <v>8</v>
-      </c>
       <c r="X2">
-        <v>192</v>
+        <v>135</v>
       </c>
       <c r="Y2" t="s">
+        <v>85</v>
+      </c>
+      <c r="Z2" t="s">
         <v>86</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>87</v>
       </c>
       <c r="AC2" t="s">
         <v>80</v>
       </c>
       <c r="AD2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" t="s">
-        <v>76</v>
-      </c>
-      <c r="K3" t="s">
-        <v>77</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="N3" t="s">
-        <v>78</v>
-      </c>
-      <c r="O3">
-        <v>1</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <v>2026</v>
-      </c>
-      <c r="S3" t="s">
-        <v>79</v>
-      </c>
-      <c r="T3">
-        <v>2</v>
-      </c>
-      <c r="U3">
-        <v>7</v>
-      </c>
-      <c r="V3">
-        <v>1</v>
-      </c>
-      <c r="W3">
-        <v>8</v>
-      </c>
-      <c r="X3">
-        <v>80</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD3" t="s">
         <v>81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Attach to existing Chrome instance for eGramSwaraj bot
- Updated workflow to connect to a running Chrome instance with remote debugging instead of launching a new one.
- Implemented _attach_to_chrome function to reuse existing browser context and page.
- Removed browser launch code and adjusted logging messages to reflect the new connection method.
- Ensured that the Chrome instance remains open after the bot's execution.
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Automation\egram_bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A741823A-05DE-4C25-9AD9-95FCC88A0145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835A7525-C62C-48ED-AD1A-C9183534F0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="167">
   <si>
     <t>Activity_Key</t>
   </si>
@@ -289,6 +289,246 @@
   </si>
   <si>
     <t>Matsaya Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0280</t>
+  </si>
+  <si>
+    <t>Theme 7 - Socially Just and Socially Secured Village</t>
+  </si>
+  <si>
+    <t>Awareness on Discrimination against SC/ST/PVTG/religious minority communities (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Welfare of the weaker sections</t>
+  </si>
+  <si>
+    <t>Mahatma Gandhi National Rural Employment Guarantee Scheme (MGNREGS) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Department of Food &amp; Public Distribution</t>
+  </si>
+  <si>
+    <t>ACT-0281</t>
+  </si>
+  <si>
+    <t>Awareness Campaign about UDID</t>
+  </si>
+  <si>
+    <t>Social welfare</t>
+  </si>
+  <si>
+    <t>Deendayal Upadhyaya Grameen Kaushalya Yojana(DDUGKY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Department of Health &amp; Family Welfare</t>
+  </si>
+  <si>
+    <t>ACT-0282</t>
+  </si>
+  <si>
+    <t>Awareness Campaign on Scheme related to pension</t>
+  </si>
+  <si>
+    <t>National Social Assistance Programme (NSAP) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Ministry of Women and Child Development</t>
+  </si>
+  <si>
+    <t>ACT-0283</t>
+  </si>
+  <si>
+    <t>Awareness Campaign on different social protection scheme</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri AwasYojana Gramin PMAY (G) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Ministry of Power</t>
+  </si>
+  <si>
+    <t>ACT-0284</t>
+  </si>
+  <si>
+    <t>Awareness on Discrimination against transgenders (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Swachh Bharat Mission (Gramin) (SBM (G)] - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0285</t>
+  </si>
+  <si>
+    <t>Awareness on Issues related to migrant labourers (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Jal Jeevan Mission (JJM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0286</t>
+  </si>
+  <si>
+    <t>Awareness on Issues related to persons with disabilities (PWDs) (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Deendayal Upadhyaya Gram Jyoti Yojana (DDUGJY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Department of Rural Development</t>
+  </si>
+  <si>
+    <t>ACT-0287</t>
+  </si>
+  <si>
+    <t>Awareness on Issues related to sanitation workers (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Department of Drinking Water and Sanitation</t>
+  </si>
+  <si>
+    <t>ACT-0288</t>
+  </si>
+  <si>
+    <t>Awareness on Issues related to sex workers (Social exclusion)</t>
+  </si>
+  <si>
+    <t>National Health Mission (NHM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0289</t>
+  </si>
+  <si>
+    <t>Awareness on Issues related to single women/widows (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Mid-Day Meal Scheme (MDM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0290</t>
+  </si>
+  <si>
+    <t>Awareness on Issues related to the elderly (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Matru Vandana Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0291</t>
+  </si>
+  <si>
+    <t>Awareness on Lack of access to education for Persons with Disabilities (Inclusive Education)</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Ujjwala Yojana - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0292</t>
+  </si>
+  <si>
+    <t>Awareness on Witch Hunting (Social exclusion)</t>
+  </si>
+  <si>
+    <t>Antodaya Anna Yojana - Center Scheme</t>
+  </si>
+  <si>
+    <t>Conduct IEC/awareness and  inclusion camps for social protection and beneficiary-oriented schemes</t>
+  </si>
+  <si>
+    <t>Conduct IEC/awareness and inclusion camps for social protection and beneficiary-oriented schemes</t>
+  </si>
+  <si>
+    <t>Samagara Shikha Abhiyan - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0002</t>
+  </si>
+  <si>
+    <t>Create awareness on FPOs and support formation/strngthening of FPOs through farmer mobilisation</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
+    <t>Poshan Abhiyan/ICDS - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0003</t>
+  </si>
+  <si>
+    <t>Create awareness on volunteering and community support initiatices, including animal welfare activities</t>
+  </si>
+  <si>
+    <t>Animal husbandry</t>
+  </si>
+  <si>
+    <t>Beti Bachao Beti Padao - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0015</t>
+  </si>
+  <si>
+    <t>Facilitate formation oh SHGs and provide support for strengthening SHGs in Gram Panchayats</t>
+  </si>
+  <si>
+    <t>National Rural Livelihood Mission (NRLM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0020</t>
+  </si>
+  <si>
+    <t>Facilitation/provision of skill development training</t>
+  </si>
+  <si>
+    <t>Technical training and vocational education</t>
+  </si>
+  <si>
+    <t>Beneficiary Oriented Programmes</t>
+  </si>
+  <si>
+    <t>Pashudhan Scheme - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0036</t>
+  </si>
+  <si>
+    <t>Theme 2 - Healthy Village</t>
+  </si>
+  <si>
+    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of Vector Borne Diseases (VBD)</t>
+  </si>
+  <si>
+    <t>Health</t>
+  </si>
+  <si>
+    <t>Janani Surakha Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0037</t>
+  </si>
+  <si>
+    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of anaemia; vicious cycle of anaemia</t>
+  </si>
+  <si>
+    <t>Ayushman Bharat - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0043</t>
+  </si>
+  <si>
+    <t>Oraginizing awareness camp/ program on significance of health &amp; nutrition</t>
+  </si>
+  <si>
+    <t>Family welfare</t>
+  </si>
+  <si>
+    <t>National Biogas and Manure Management Programme - Center Scheme</t>
   </si>
 </sst>
 </file>
@@ -322,7 +562,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -332,12 +572,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFED7D31"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -364,7 +598,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,7 +901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG2"/>
+  <dimension ref="A1:AG23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -807,22 +1041,25 @@
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
         <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>85</v>
+        <v>89</v>
+      </c>
+      <c r="G2" t="s">
+        <v>78</v>
       </c>
       <c r="I2" t="s">
         <v>76</v>
@@ -852,30 +1089,1650 @@
         <v>79</v>
       </c>
       <c r="T2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V2">
         <v>5</v>
       </c>
       <c r="W2">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="X2">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="Y2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Z2" t="s">
-        <v>86</v>
+        <v>91</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>92</v>
       </c>
       <c r="AC2" t="s">
         <v>80</v>
       </c>
       <c r="AD2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" t="s">
+        <v>76</v>
+      </c>
+      <c r="K3" t="s">
+        <v>77</v>
+      </c>
+      <c r="N3" t="s">
+        <v>78</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>2026</v>
+      </c>
+      <c r="S3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T3">
+        <v>7</v>
+      </c>
+      <c r="U3">
+        <v>1</v>
+      </c>
+      <c r="V3">
+        <v>1</v>
+      </c>
+      <c r="W3">
+        <v>6</v>
+      </c>
+      <c r="X3">
+        <v>54</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G4" t="s">
+        <v>78</v>
+      </c>
+      <c r="I4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J4" t="s">
+        <v>76</v>
+      </c>
+      <c r="K4" t="s">
+        <v>77</v>
+      </c>
+      <c r="N4" t="s">
+        <v>78</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>2026</v>
+      </c>
+      <c r="S4" t="s">
+        <v>79</v>
+      </c>
+      <c r="T4">
+        <v>8</v>
+      </c>
+      <c r="U4">
+        <v>7</v>
+      </c>
+      <c r="V4">
+        <v>1</v>
+      </c>
+      <c r="W4">
+        <v>5</v>
+      </c>
+      <c r="X4">
+        <v>80</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>100</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" t="s">
+        <v>103</v>
+      </c>
+      <c r="I5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K5" t="s">
+        <v>77</v>
+      </c>
+      <c r="N5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>2026</v>
+      </c>
+      <c r="S5" t="s">
+        <v>79</v>
+      </c>
+      <c r="T5">
+        <v>2</v>
+      </c>
+      <c r="U5">
+        <v>4</v>
+      </c>
+      <c r="V5">
+        <v>9</v>
+      </c>
+      <c r="W5">
+        <v>8</v>
+      </c>
+      <c r="X5">
+        <v>120</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>104</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>105</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" t="s">
+        <v>107</v>
+      </c>
+      <c r="G6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I6" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" t="s">
+        <v>76</v>
+      </c>
+      <c r="K6" t="s">
+        <v>77</v>
+      </c>
+      <c r="N6" t="s">
+        <v>78</v>
+      </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>2026</v>
+      </c>
+      <c r="S6" t="s">
+        <v>79</v>
+      </c>
+      <c r="T6">
+        <v>6</v>
+      </c>
+      <c r="U6">
+        <v>10</v>
+      </c>
+      <c r="V6">
+        <v>5</v>
+      </c>
+      <c r="W6">
+        <v>2</v>
+      </c>
+      <c r="X6">
+        <v>42</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>108</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G7" t="s">
+        <v>78</v>
+      </c>
+      <c r="I7" t="s">
+        <v>76</v>
+      </c>
+      <c r="J7" t="s">
+        <v>76</v>
+      </c>
+      <c r="K7" t="s">
+        <v>77</v>
+      </c>
+      <c r="N7" t="s">
+        <v>78</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>2026</v>
+      </c>
+      <c r="S7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T7">
+        <v>10</v>
+      </c>
+      <c r="U7">
+        <v>8</v>
+      </c>
+      <c r="V7">
+        <v>4</v>
+      </c>
+      <c r="W7">
+        <v>5</v>
+      </c>
+      <c r="X7">
+        <v>110</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>111</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" t="s">
+        <v>113</v>
+      </c>
+      <c r="G8" t="s">
+        <v>78</v>
+      </c>
+      <c r="I8" t="s">
+        <v>76</v>
+      </c>
+      <c r="J8" t="s">
+        <v>76</v>
+      </c>
+      <c r="K8" t="s">
+        <v>77</v>
+      </c>
+      <c r="N8" t="s">
+        <v>78</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>2026</v>
+      </c>
+      <c r="S8" t="s">
+        <v>79</v>
+      </c>
+      <c r="T8">
+        <v>5</v>
+      </c>
+      <c r="U8">
+        <v>3</v>
+      </c>
+      <c r="V8">
+        <v>1</v>
+      </c>
+      <c r="W8">
+        <v>8</v>
+      </c>
+      <c r="X8">
+        <v>72</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>113</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>115</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" t="s">
+        <v>117</v>
+      </c>
+      <c r="G9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s">
+        <v>76</v>
+      </c>
+      <c r="K9" t="s">
+        <v>77</v>
+      </c>
+      <c r="N9" t="s">
+        <v>78</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>2026</v>
+      </c>
+      <c r="S9" t="s">
+        <v>79</v>
+      </c>
+      <c r="T9">
+        <v>6</v>
+      </c>
+      <c r="U9">
+        <v>4</v>
+      </c>
+      <c r="V9">
+        <v>4</v>
+      </c>
+      <c r="W9">
+        <v>9</v>
+      </c>
+      <c r="X9">
+        <v>126</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>117</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>118</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>119</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" t="s">
+        <v>121</v>
+      </c>
+      <c r="G10" t="s">
+        <v>78</v>
+      </c>
+      <c r="I10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" t="s">
+        <v>76</v>
+      </c>
+      <c r="K10" t="s">
+        <v>77</v>
+      </c>
+      <c r="N10" t="s">
+        <v>78</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>2026</v>
+      </c>
+      <c r="S10" t="s">
+        <v>79</v>
+      </c>
+      <c r="T10">
+        <v>10</v>
+      </c>
+      <c r="U10">
+        <v>8</v>
+      </c>
+      <c r="V10">
+        <v>8</v>
+      </c>
+      <c r="W10">
+        <v>7</v>
+      </c>
+      <c r="X10">
+        <v>182</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>121</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" t="s">
+        <v>124</v>
+      </c>
+      <c r="G11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" t="s">
+        <v>76</v>
+      </c>
+      <c r="J11" t="s">
+        <v>76</v>
+      </c>
+      <c r="K11" t="s">
+        <v>77</v>
+      </c>
+      <c r="N11" t="s">
+        <v>78</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>2026</v>
+      </c>
+      <c r="S11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T11">
+        <v>2</v>
+      </c>
+      <c r="U11">
+        <v>5</v>
+      </c>
+      <c r="V11">
+        <v>4</v>
+      </c>
+      <c r="W11">
+        <v>4</v>
+      </c>
+      <c r="X11">
+        <v>44</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>125</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12" t="s">
+        <v>88</v>
+      </c>
+      <c r="C12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12" t="s">
+        <v>76</v>
+      </c>
+      <c r="K12" t="s">
+        <v>77</v>
+      </c>
+      <c r="N12" t="s">
+        <v>78</v>
+      </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>2026</v>
+      </c>
+      <c r="S12" t="s">
+        <v>79</v>
+      </c>
+      <c r="T12">
+        <v>7</v>
+      </c>
+      <c r="U12">
+        <v>4</v>
+      </c>
+      <c r="V12">
+        <v>1</v>
+      </c>
+      <c r="W12">
+        <v>1</v>
+      </c>
+      <c r="X12">
+        <v>12</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>127</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" t="s">
+        <v>130</v>
+      </c>
+      <c r="D13" t="s">
+        <v>131</v>
+      </c>
+      <c r="E13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" t="s">
+        <v>130</v>
+      </c>
+      <c r="G13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" t="s">
+        <v>76</v>
+      </c>
+      <c r="K13" t="s">
+        <v>77</v>
+      </c>
+      <c r="N13" t="s">
+        <v>78</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>2026</v>
+      </c>
+      <c r="S13" t="s">
+        <v>79</v>
+      </c>
+      <c r="T13">
+        <v>5</v>
+      </c>
+      <c r="U13">
+        <v>3</v>
+      </c>
+      <c r="V13">
+        <v>1</v>
+      </c>
+      <c r="W13">
+        <v>7</v>
+      </c>
+      <c r="X13">
+        <v>63</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>130</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>132</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>115</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" t="s">
+        <v>95</v>
+      </c>
+      <c r="E14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" t="s">
+        <v>134</v>
+      </c>
+      <c r="G14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" t="s">
+        <v>76</v>
+      </c>
+      <c r="J14" t="s">
+        <v>76</v>
+      </c>
+      <c r="K14" t="s">
+        <v>77</v>
+      </c>
+      <c r="N14" t="s">
+        <v>78</v>
+      </c>
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>2026</v>
+      </c>
+      <c r="S14" t="s">
+        <v>79</v>
+      </c>
+      <c r="T14">
+        <v>5</v>
+      </c>
+      <c r="U14">
+        <v>2</v>
+      </c>
+      <c r="V14">
+        <v>3</v>
+      </c>
+      <c r="W14">
+        <v>5</v>
+      </c>
+      <c r="X14">
+        <v>50</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>134</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>135</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" t="s">
+        <v>137</v>
+      </c>
+      <c r="I15" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" t="s">
+        <v>76</v>
+      </c>
+      <c r="K15" t="s">
+        <v>77</v>
+      </c>
+      <c r="N15" t="s">
+        <v>78</v>
+      </c>
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>2026</v>
+      </c>
+      <c r="S15" t="s">
+        <v>79</v>
+      </c>
+      <c r="T15">
+        <v>3</v>
+      </c>
+      <c r="U15">
+        <v>8</v>
+      </c>
+      <c r="V15">
+        <v>8</v>
+      </c>
+      <c r="W15">
+        <v>10</v>
+      </c>
+      <c r="X15">
+        <v>190</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>136</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>138</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>139</v>
+      </c>
+      <c r="B16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D16" t="s">
+        <v>141</v>
+      </c>
+      <c r="E16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" t="s">
+        <v>140</v>
+      </c>
+      <c r="I16" t="s">
+        <v>76</v>
+      </c>
+      <c r="J16" t="s">
+        <v>76</v>
+      </c>
+      <c r="K16" t="s">
+        <v>77</v>
+      </c>
+      <c r="N16" t="s">
+        <v>78</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>2026</v>
+      </c>
+      <c r="S16" t="s">
+        <v>79</v>
+      </c>
+      <c r="T16">
+        <v>8</v>
+      </c>
+      <c r="U16">
+        <v>4</v>
+      </c>
+      <c r="V16">
+        <v>4</v>
+      </c>
+      <c r="W16">
+        <v>5</v>
+      </c>
+      <c r="X16">
+        <v>80</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>140</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>142</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D17" t="s">
+        <v>145</v>
+      </c>
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" t="s">
+        <v>144</v>
+      </c>
+      <c r="G17" t="s">
+        <v>78</v>
+      </c>
+      <c r="I17" t="s">
+        <v>76</v>
+      </c>
+      <c r="J17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K17" t="s">
+        <v>77</v>
+      </c>
+      <c r="N17" t="s">
+        <v>78</v>
+      </c>
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>2026</v>
+      </c>
+      <c r="S17" t="s">
+        <v>79</v>
+      </c>
+      <c r="T17">
+        <v>3</v>
+      </c>
+      <c r="U17">
+        <v>8</v>
+      </c>
+      <c r="V17">
+        <v>8</v>
+      </c>
+      <c r="W17">
+        <v>7</v>
+      </c>
+      <c r="X17">
+        <v>133</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>146</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" t="s">
+        <v>148</v>
+      </c>
+      <c r="I18" t="s">
+        <v>76</v>
+      </c>
+      <c r="J18" t="s">
+        <v>76</v>
+      </c>
+      <c r="K18" t="s">
+        <v>77</v>
+      </c>
+      <c r="N18" t="s">
+        <v>78</v>
+      </c>
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>2026</v>
+      </c>
+      <c r="S18" t="s">
+        <v>79</v>
+      </c>
+      <c r="T18">
+        <v>9</v>
+      </c>
+      <c r="U18">
+        <v>6</v>
+      </c>
+      <c r="V18">
+        <v>6</v>
+      </c>
+      <c r="W18">
+        <v>10</v>
+      </c>
+      <c r="X18">
+        <v>210</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>148</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>149</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E19" t="s">
+        <v>153</v>
+      </c>
+      <c r="F19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G19" t="s">
+        <v>78</v>
+      </c>
+      <c r="I19" t="s">
+        <v>76</v>
+      </c>
+      <c r="J19" t="s">
+        <v>76</v>
+      </c>
+      <c r="K19" t="s">
+        <v>77</v>
+      </c>
+      <c r="N19" t="s">
+        <v>78</v>
+      </c>
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>2026</v>
+      </c>
+      <c r="S19" t="s">
+        <v>79</v>
+      </c>
+      <c r="T19">
+        <v>1</v>
+      </c>
+      <c r="U19">
+        <v>2</v>
+      </c>
+      <c r="V19">
+        <v>8</v>
+      </c>
+      <c r="W19">
+        <v>7</v>
+      </c>
+      <c r="X19">
+        <v>77</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>151</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>154</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" t="s">
+        <v>85</v>
+      </c>
+      <c r="I20" t="s">
+        <v>76</v>
+      </c>
+      <c r="J20" t="s">
+        <v>76</v>
+      </c>
+      <c r="K20" t="s">
+        <v>77</v>
+      </c>
+      <c r="N20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>2026</v>
+      </c>
+      <c r="S20" t="s">
+        <v>79</v>
+      </c>
+      <c r="T20">
+        <v>7</v>
+      </c>
+      <c r="U20">
+        <v>3</v>
+      </c>
+      <c r="V20">
+        <v>5</v>
+      </c>
+      <c r="W20">
+        <v>9</v>
+      </c>
+      <c r="X20">
+        <v>135</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>85</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>86</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" t="s">
+        <v>156</v>
+      </c>
+      <c r="C21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D21" t="s">
+        <v>158</v>
+      </c>
+      <c r="E21" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" t="s">
+        <v>157</v>
+      </c>
+      <c r="I21" t="s">
+        <v>76</v>
+      </c>
+      <c r="J21" t="s">
+        <v>76</v>
+      </c>
+      <c r="K21" t="s">
+        <v>77</v>
+      </c>
+      <c r="N21" t="s">
+        <v>78</v>
+      </c>
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>2026</v>
+      </c>
+      <c r="S21" t="s">
+        <v>79</v>
+      </c>
+      <c r="T21">
+        <v>6</v>
+      </c>
+      <c r="U21">
+        <v>1</v>
+      </c>
+      <c r="V21">
+        <v>6</v>
+      </c>
+      <c r="W21">
+        <v>9</v>
+      </c>
+      <c r="X21">
+        <v>117</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>159</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C22" t="s">
+        <v>161</v>
+      </c>
+      <c r="D22" t="s">
+        <v>158</v>
+      </c>
+      <c r="E22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" t="s">
+        <v>161</v>
+      </c>
+      <c r="G22" t="s">
+        <v>78</v>
+      </c>
+      <c r="I22" t="s">
+        <v>76</v>
+      </c>
+      <c r="J22" t="s">
+        <v>76</v>
+      </c>
+      <c r="K22" t="s">
+        <v>77</v>
+      </c>
+      <c r="N22" t="s">
+        <v>78</v>
+      </c>
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>2026</v>
+      </c>
+      <c r="S22" t="s">
+        <v>79</v>
+      </c>
+      <c r="T22">
+        <v>7</v>
+      </c>
+      <c r="U22">
+        <v>4</v>
+      </c>
+      <c r="V22">
+        <v>7</v>
+      </c>
+      <c r="W22">
+        <v>6</v>
+      </c>
+      <c r="X22">
+        <v>108</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>161</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>163</v>
+      </c>
+      <c r="B23" t="s">
+        <v>156</v>
+      </c>
+      <c r="C23" t="s">
+        <v>164</v>
+      </c>
+      <c r="D23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" t="s">
+        <v>164</v>
+      </c>
+      <c r="G23" t="s">
+        <v>78</v>
+      </c>
+      <c r="I23" t="s">
+        <v>76</v>
+      </c>
+      <c r="J23" t="s">
+        <v>76</v>
+      </c>
+      <c r="K23" t="s">
+        <v>77</v>
+      </c>
+      <c r="N23" t="s">
+        <v>78</v>
+      </c>
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>2026</v>
+      </c>
+      <c r="S23" t="s">
+        <v>79</v>
+      </c>
+      <c r="T23">
+        <v>9</v>
+      </c>
+      <c r="U23">
+        <v>8</v>
+      </c>
+      <c r="V23">
+        <v>4</v>
+      </c>
+      <c r="W23">
+        <v>1</v>
+      </c>
+      <c r="X23">
+        <v>21</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>164</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>166</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD23" t="s">
         <v>81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor activity output handling and form filler logic
- Simplified the radio button click handling in StructuredModalOutputHandler to ensure the native click executes the portal's inline onclick only once, preventing re-validation and modal hiding.
- Removed redundant event dispatching in select_start_month function to streamline the selection process.
- Introduced ensure_start_month_ready function to validate the selected month before dependent validation, improving reliability in form filling.
- Updated FormFiller to call ensure_start_month_ready before processing activity output, ensuring the persisted value is accurate after AJAX updates.
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Automation\egram_bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835A7525-C62C-48ED-AD1A-C9183534F0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D7A009-1574-4826-BDC8-7CEC3E5069FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,14 +21,14 @@
     <sheet name="Asset" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Activities!$A$1:$AG$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Activities!$A$1:$AG$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="162">
   <si>
     <t>Activity_Key</t>
   </si>
@@ -276,259 +276,244 @@
     <t>Save and Forward</t>
   </si>
   <si>
+    <t>Social welfare</t>
+  </si>
+  <si>
+    <t>National Social Assistance Programme (NSAP) - Center Scheme</t>
+  </si>
+  <si>
     <t>Theme 1 - Poverty Free and Enhanced Livelihoods Village</t>
   </si>
   <si>
+    <t>Conduct IEC/awareness and inclusion camps for social protection and beneficiary-oriented schemes</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Ujjwala Yojana - Center Scheme</t>
+  </si>
+  <si>
+    <t>Matsaya Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>Janani Surakha Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>Ayushman Bharat - Center Scheme</t>
+  </si>
+  <si>
+    <t>National Biogas and Manure Management Programme - Center Scheme</t>
+  </si>
+  <si>
+    <t>Conduct IEC/awareness and  inclusion camps for social protection and beneficiary-oriented schemes</t>
+  </si>
+  <si>
+    <t>Mahatma Gandhi National Rural Employment Guarantee Scheme (MGNREGS) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Deendayal Upadhyaya Grameen Kaushalya Yojana(DDUGKY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri AwasYojana Gramin PMAY (G) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Swachh Bharat Mission (Gramin) (SBM (G)] - Center Scheme</t>
+  </si>
+  <si>
+    <t>Jal Jeevan Mission (JJM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Deendayal Upadhyaya Gram Jyoti Yojana (DDUGJY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>National Health Mission (NHM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Mid-Day Meal Scheme (MDM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Matru Vandana Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>Antodaya Anna Yojana - Center Scheme</t>
+  </si>
+  <si>
+    <t>Samagara Shikha Abhiyan - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0002</t>
+  </si>
+  <si>
+    <t>Create awareness on FPOs and support formation/strngthening of FPOs through farmer mobilisation</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
+    <t>Poshan Abhiyan/ICDS - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0003</t>
+  </si>
+  <si>
+    <t>Create awareness on volunteering and community support initiatices, including animal welfare activities</t>
+  </si>
+  <si>
+    <t>Animal husbandry</t>
+  </si>
+  <si>
+    <t>Beti Bachao Beti Padao - Center Scheme</t>
+  </si>
+  <si>
+    <t>National Rural Livelihood Mission (NRLM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Beneficiary Oriented Programmes</t>
+  </si>
+  <si>
+    <t>Pashudhan Scheme - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0036</t>
+  </si>
+  <si>
+    <t>Theme 2 - Healthy Village</t>
+  </si>
+  <si>
+    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of Vector Borne Diseases (VBD)</t>
+  </si>
+  <si>
+    <t>Health</t>
+  </si>
+  <si>
+    <t>ACT-0037</t>
+  </si>
+  <si>
+    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of anaemia; vicious cycle of anaemia</t>
+  </si>
+  <si>
+    <t>ACT-0043</t>
+  </si>
+  <si>
+    <t>Oraginizing awareness camp/ program on significance of health &amp; nutrition</t>
+  </si>
+  <si>
+    <t>Family welfare</t>
+  </si>
+  <si>
+    <t>ACT-0044</t>
+  </si>
+  <si>
+    <t>Oranizing Training of Mid Wives on safe &amp; institutional delivery</t>
+  </si>
+  <si>
+    <t>ACT-0046</t>
+  </si>
+  <si>
+    <t>Organize Mental Health Awareness Camps  &amp; Development of IEC materials on Mental Health</t>
+  </si>
+  <si>
+    <t>Organize Mental Health Awareness Camps &amp; Development of IEC materials on Mental Health</t>
+  </si>
+  <si>
+    <t>ACT-0047</t>
+  </si>
+  <si>
+    <t>Organizing Awareness &amp; IEC campaign on Health Schemes/ Program</t>
+  </si>
+  <si>
+    <t>ACT-0048</t>
+  </si>
+  <si>
+    <t>Organizing Awareness Campaign/ Program including Nukkad Natak/Street Play on Maternal and Child health</t>
+  </si>
+  <si>
+    <t>Cultural activities</t>
+  </si>
+  <si>
+    <t>ACT-0051</t>
+  </si>
+  <si>
+    <t>Organizing awareness camp about child heath through campaign</t>
+  </si>
+  <si>
+    <t>ACT-0052</t>
+  </si>
+  <si>
+    <t>Organizing awareness camp on institutional delivery and early registration to the hospitals for ante-natal chaeck up &amp; post natal check up of pregnanat mothers</t>
+  </si>
+  <si>
+    <t>ACT-0053</t>
+  </si>
+  <si>
+    <t>Organizing awareness camp on rountine immunization of children</t>
+  </si>
+  <si>
+    <t>ACT-0015</t>
+  </si>
+  <si>
+    <t>Facilitate formation oh SHGs and provide support for strengthening SHGs in Gram Panchayats</t>
+  </si>
+  <si>
     <t>Poverty allevation programme</t>
   </si>
   <si>
+    <t>ACT-0020</t>
+  </si>
+  <si>
+    <t>Facilitation/provision of skill development training</t>
+  </si>
+  <si>
+    <t>Technical training and vocational education</t>
+  </si>
+  <si>
     <t>ACT-0028</t>
   </si>
   <si>
     <t>Organise career counselling camps to promote self-employment opportunities at the GP level</t>
   </si>
   <si>
-    <t>Matsaya Yojna - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0280</t>
-  </si>
-  <si>
-    <t>Theme 7 - Socially Just and Socially Secured Village</t>
-  </si>
-  <si>
-    <t>Awareness on Discrimination against SC/ST/PVTG/religious minority communities (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Welfare of the weaker sections</t>
-  </si>
-  <si>
-    <t>Mahatma Gandhi National Rural Employment Guarantee Scheme (MGNREGS) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Department of Food &amp; Public Distribution</t>
-  </si>
-  <si>
-    <t>ACT-0281</t>
-  </si>
-  <si>
-    <t>Awareness Campaign about UDID</t>
-  </si>
-  <si>
-    <t>Social welfare</t>
-  </si>
-  <si>
-    <t>Deendayal Upadhyaya Grameen Kaushalya Yojana(DDUGKY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Department of Health &amp; Family Welfare</t>
-  </si>
-  <si>
-    <t>ACT-0282</t>
-  </si>
-  <si>
-    <t>Awareness Campaign on Scheme related to pension</t>
-  </si>
-  <si>
-    <t>National Social Assistance Programme (NSAP) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Ministry of Women and Child Development</t>
-  </si>
-  <si>
-    <t>ACT-0283</t>
-  </si>
-  <si>
-    <t>Awareness Campaign on different social protection scheme</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri AwasYojana Gramin PMAY (G) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Ministry of Power</t>
-  </si>
-  <si>
-    <t>ACT-0284</t>
-  </si>
-  <si>
-    <t>Awareness on Discrimination against transgenders (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Swachh Bharat Mission (Gramin) (SBM (G)] - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0285</t>
-  </si>
-  <si>
-    <t>Awareness on Issues related to migrant labourers (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Jal Jeevan Mission (JJM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0286</t>
-  </si>
-  <si>
-    <t>Awareness on Issues related to persons with disabilities (PWDs) (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Deendayal Upadhyaya Gram Jyoti Yojana (DDUGJY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Department of Rural Development</t>
-  </si>
-  <si>
-    <t>ACT-0287</t>
-  </si>
-  <si>
-    <t>Awareness on Issues related to sanitation workers (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Department of Drinking Water and Sanitation</t>
-  </si>
-  <si>
-    <t>ACT-0288</t>
-  </si>
-  <si>
-    <t>Awareness on Issues related to sex workers (Social exclusion)</t>
-  </si>
-  <si>
-    <t>National Health Mission (NHM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0289</t>
-  </si>
-  <si>
-    <t>Awareness on Issues related to single women/widows (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Mid-Day Meal Scheme (MDM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0290</t>
-  </si>
-  <si>
-    <t>Awareness on Issues related to the elderly (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Matru Vandana Yojna - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0291</t>
-  </si>
-  <si>
-    <t>Awareness on Lack of access to education for Persons with Disabilities (Inclusive Education)</t>
-  </si>
-  <si>
-    <t>Education</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Ujjwala Yojana - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0292</t>
-  </si>
-  <si>
-    <t>Awareness on Witch Hunting (Social exclusion)</t>
-  </si>
-  <si>
-    <t>Antodaya Anna Yojana - Center Scheme</t>
-  </si>
-  <si>
-    <t>Conduct IEC/awareness and  inclusion camps for social protection and beneficiary-oriented schemes</t>
-  </si>
-  <si>
-    <t>Conduct IEC/awareness and inclusion camps for social protection and beneficiary-oriented schemes</t>
-  </si>
-  <si>
-    <t>Samagara Shikha Abhiyan - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0002</t>
-  </si>
-  <si>
-    <t>Create awareness on FPOs and support formation/strngthening of FPOs through farmer mobilisation</t>
-  </si>
-  <si>
-    <t>Agriculture</t>
-  </si>
-  <si>
-    <t>Poshan Abhiyan/ICDS - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0003</t>
-  </si>
-  <si>
-    <t>Create awareness on volunteering and community support initiatices, including animal welfare activities</t>
-  </si>
-  <si>
-    <t>Animal husbandry</t>
-  </si>
-  <si>
-    <t>Beti Bachao Beti Padao - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0015</t>
-  </si>
-  <si>
-    <t>Facilitate formation oh SHGs and provide support for strengthening SHGs in Gram Panchayats</t>
-  </si>
-  <si>
-    <t>National Rural Livelihood Mission (NRLM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0020</t>
-  </si>
-  <si>
-    <t>Facilitation/provision of skill development training</t>
-  </si>
-  <si>
-    <t>Technical training and vocational education</t>
-  </si>
-  <si>
-    <t>Beneficiary Oriented Programmes</t>
-  </si>
-  <si>
-    <t>Pashudhan Scheme - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0036</t>
-  </si>
-  <si>
-    <t>Theme 2 - Healthy Village</t>
-  </si>
-  <si>
-    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of Vector Borne Diseases (VBD)</t>
-  </si>
-  <si>
-    <t>Health</t>
-  </si>
-  <si>
-    <t>Janani Surakha Yojna - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0037</t>
-  </si>
-  <si>
-    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of anaemia; vicious cycle of anaemia</t>
-  </si>
-  <si>
-    <t>Ayushman Bharat - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0043</t>
-  </si>
-  <si>
-    <t>Oraginizing awareness camp/ program on significance of health &amp; nutrition</t>
-  </si>
-  <si>
-    <t>Family welfare</t>
-  </si>
-  <si>
-    <t>National Biogas and Manure Management Programme - Center Scheme</t>
+    <t>ACT-0306</t>
+  </si>
+  <si>
+    <t>Theme 8 - Village with Good Governance</t>
+  </si>
+  <si>
+    <t>Capacity Building &amp; Training of Elected Representatives, Functionaries &amp; other stakeholders</t>
+  </si>
+  <si>
+    <t>ACT-0310</t>
+  </si>
+  <si>
+    <t>Cost for Disaster Readiness, relief and mitigation activities (Training, planning, survey etc)</t>
+  </si>
+  <si>
+    <t>Adult and non-formal education</t>
+  </si>
+  <si>
+    <t>ACT-0313</t>
+  </si>
+  <si>
+    <t>IEC &amp; Awareness Campaign for active participation in Gram Sabha, Ward Sabha, Mahila Sabha</t>
+  </si>
+  <si>
+    <t>ACT-0314</t>
+  </si>
+  <si>
+    <t>IEC &amp; Awareness campaign on SHG-PRI Convergence /Public Services/ Service Delivery Provisions/ RTI/Grivences</t>
+  </si>
+  <si>
+    <t>ACT-0315</t>
+  </si>
+  <si>
+    <t>IEC &amp; Awareness on disaster preparedness and mitigation</t>
+  </si>
+  <si>
+    <t>ACT-0317</t>
+  </si>
+  <si>
+    <t>Organising of Gram Sabha/ Ward Sabha/ Mahila Sabha/ GPDP</t>
   </si>
 </sst>
 </file>
@@ -587,7 +572,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -598,7 +583,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1040,26 +1024,23 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>87</v>
+      <c r="A2" t="s">
+        <v>148</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>150</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="E2" t="s">
         <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" t="s">
-        <v>78</v>
+        <v>150</v>
       </c>
       <c r="I2" t="s">
         <v>76</v>
@@ -1092,24 +1073,21 @@
         <v>8</v>
       </c>
       <c r="U2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V2">
         <v>5</v>
       </c>
       <c r="W2">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="X2">
-        <v>60</v>
+        <v>153</v>
       </c>
       <c r="Y2" t="s">
-        <v>89</v>
+        <v>150</v>
       </c>
       <c r="Z2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA2" t="s">
         <v>92</v>
       </c>
       <c r="AC2" t="s">
@@ -1121,22 +1099,22 @@
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>151</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>153</v>
       </c>
       <c r="E3" t="s">
         <v>75</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="I3" t="s">
         <v>76</v>
@@ -1166,28 +1144,25 @@
         <v>79</v>
       </c>
       <c r="T3">
+        <v>5</v>
+      </c>
+      <c r="U3">
         <v>7</v>
       </c>
-      <c r="U3">
-        <v>1</v>
-      </c>
       <c r="V3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="W3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="X3">
-        <v>54</v>
+        <v>198</v>
       </c>
       <c r="Y3" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="Z3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="AC3" t="s">
         <v>80</v>
@@ -1198,25 +1173,22 @@
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>154</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
         <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G4" t="s">
-        <v>78</v>
+        <v>155</v>
       </c>
       <c r="I4" t="s">
         <v>76</v>
@@ -1246,28 +1218,25 @@
         <v>79</v>
       </c>
       <c r="T4">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="U4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V4">
+        <v>3</v>
+      </c>
+      <c r="W4">
         <v>1</v>
       </c>
-      <c r="W4">
-        <v>5</v>
-      </c>
       <c r="X4">
-        <v>80</v>
+        <v>11</v>
       </c>
       <c r="Y4" t="s">
-        <v>99</v>
+        <v>155</v>
       </c>
       <c r="Z4" t="s">
-        <v>100</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="AC4" t="s">
         <v>80</v>
@@ -1278,22 +1247,22 @@
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>156</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>157</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>153</v>
       </c>
       <c r="E5" t="s">
         <v>75</v>
       </c>
       <c r="F5" t="s">
-        <v>103</v>
+        <v>157</v>
       </c>
       <c r="I5" t="s">
         <v>76</v>
@@ -1323,28 +1292,25 @@
         <v>79</v>
       </c>
       <c r="T5">
+        <v>6</v>
+      </c>
+      <c r="U5">
+        <v>8</v>
+      </c>
+      <c r="V5">
+        <v>3</v>
+      </c>
+      <c r="W5">
         <v>2</v>
       </c>
-      <c r="U5">
-        <v>4</v>
-      </c>
-      <c r="V5">
-        <v>9</v>
-      </c>
-      <c r="W5">
-        <v>8</v>
-      </c>
       <c r="X5">
-        <v>120</v>
+        <v>34</v>
       </c>
       <c r="Y5" t="s">
-        <v>103</v>
+        <v>157</v>
       </c>
       <c r="Z5" t="s">
-        <v>104</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="AC5" t="s">
         <v>80</v>
@@ -1355,25 +1321,22 @@
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>159</v>
       </c>
       <c r="D6" t="s">
-        <v>95</v>
+        <v>153</v>
       </c>
       <c r="E6" t="s">
         <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>107</v>
-      </c>
-      <c r="G6" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="I6" t="s">
         <v>76</v>
@@ -1403,25 +1366,25 @@
         <v>79</v>
       </c>
       <c r="T6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U6">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="V6">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="W6">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="X6">
-        <v>42</v>
+        <v>160</v>
       </c>
       <c r="Y6" t="s">
-        <v>107</v>
+        <v>159</v>
       </c>
       <c r="Z6" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="AC6" t="s">
         <v>80</v>
@@ -1432,25 +1395,22 @@
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>160</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s">
-        <v>110</v>
+        <v>161</v>
       </c>
       <c r="D7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
         <v>75</v>
       </c>
       <c r="F7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G7" t="s">
-        <v>78</v>
+        <v>161</v>
       </c>
       <c r="I7" t="s">
         <v>76</v>
@@ -1480,25 +1440,25 @@
         <v>79</v>
       </c>
       <c r="T7">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U7">
         <v>8</v>
       </c>
       <c r="V7">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="W7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X7">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="Y7" t="s">
-        <v>110</v>
+        <v>161</v>
       </c>
       <c r="Z7" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="AC7" t="s">
         <v>80</v>
@@ -1509,25 +1469,22 @@
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>112</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C8" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="D8" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="E8" t="s">
         <v>75</v>
       </c>
       <c r="F8" t="s">
-        <v>113</v>
-      </c>
-      <c r="G8" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="I8" t="s">
         <v>76</v>
@@ -1557,28 +1514,25 @@
         <v>79</v>
       </c>
       <c r="T8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U8">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V8">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="W8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="X8">
-        <v>72</v>
+        <v>230</v>
       </c>
       <c r="Y8" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="Z8" t="s">
-        <v>114</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AC8" t="s">
         <v>80</v>
@@ -1589,25 +1543,22 @@
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="E9" t="s">
         <v>75</v>
       </c>
       <c r="F9" t="s">
-        <v>117</v>
-      </c>
-      <c r="G9" t="s">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="I9" t="s">
         <v>76</v>
@@ -1637,28 +1588,25 @@
         <v>79</v>
       </c>
       <c r="T9">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="U9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V9">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="W9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X9">
-        <v>126</v>
+        <v>230</v>
       </c>
       <c r="Y9" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="Z9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="AC9" t="s">
         <v>80</v>
@@ -1669,22 +1617,22 @@
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="D10" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="E10" t="s">
         <v>75</v>
       </c>
       <c r="F10" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="G10" t="s">
         <v>78</v>
@@ -1717,28 +1665,25 @@
         <v>79</v>
       </c>
       <c r="T10">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U10">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V10">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="X10">
-        <v>182</v>
+        <v>50</v>
       </c>
       <c r="Y10" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="Z10" t="s">
-        <v>122</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AC10" t="s">
         <v>80</v>
@@ -1749,25 +1694,22 @@
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="B11" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>142</v>
       </c>
       <c r="E11" t="s">
         <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>124</v>
-      </c>
-      <c r="G11" t="s">
-        <v>78</v>
+        <v>141</v>
       </c>
       <c r="I11" t="s">
         <v>76</v>
@@ -1797,25 +1739,25 @@
         <v>79</v>
       </c>
       <c r="T11">
+        <v>7</v>
+      </c>
+      <c r="U11">
+        <v>1</v>
+      </c>
+      <c r="V11">
         <v>2</v>
       </c>
-      <c r="U11">
-        <v>5</v>
-      </c>
-      <c r="V11">
-        <v>4</v>
-      </c>
       <c r="W11">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="X11">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="Y11" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="Z11" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="AC11" t="s">
         <v>80</v>
@@ -1826,22 +1768,22 @@
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="E12" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="F12" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="G12" t="s">
         <v>78</v>
@@ -1874,25 +1816,25 @@
         <v>79</v>
       </c>
       <c r="T12">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="U12">
+        <v>9</v>
+      </c>
+      <c r="V12">
         <v>4</v>
       </c>
-      <c r="V12">
-        <v>1</v>
-      </c>
       <c r="W12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X12">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="Y12" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="Z12" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="AC12" t="s">
         <v>80</v>
@@ -1903,25 +1845,22 @@
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="E13" t="s">
         <v>75</v>
       </c>
       <c r="F13" t="s">
-        <v>130</v>
-      </c>
-      <c r="G13" t="s">
-        <v>78</v>
+        <v>147</v>
       </c>
       <c r="I13" t="s">
         <v>76</v>
@@ -1951,28 +1890,25 @@
         <v>79</v>
       </c>
       <c r="T13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V13">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="W13">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="X13">
-        <v>63</v>
+        <v>150</v>
       </c>
       <c r="Y13" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="Z13" t="s">
-        <v>132</v>
-      </c>
-      <c r="AA13" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="AC13" t="s">
         <v>80</v>
@@ -1983,25 +1919,22 @@
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="D14" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="E14" t="s">
         <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>134</v>
-      </c>
-      <c r="G14" t="s">
-        <v>78</v>
+        <v>117</v>
       </c>
       <c r="I14" t="s">
         <v>76</v>
@@ -2031,25 +1964,25 @@
         <v>79</v>
       </c>
       <c r="T14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U14">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="V14">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="W14">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="X14">
-        <v>50</v>
+        <v>176</v>
       </c>
       <c r="Y14" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="Z14" t="s">
-        <v>135</v>
+        <v>102</v>
       </c>
       <c r="AC14" t="s">
         <v>80</v>
@@ -2060,22 +1993,25 @@
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C15" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
         <v>75</v>
       </c>
       <c r="F15" t="s">
-        <v>137</v>
+        <v>120</v>
+      </c>
+      <c r="G15" t="s">
+        <v>78</v>
       </c>
       <c r="I15" t="s">
         <v>76</v>
@@ -2105,25 +2041,25 @@
         <v>79</v>
       </c>
       <c r="T15">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="U15">
         <v>8</v>
       </c>
       <c r="V15">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W15">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="X15">
-        <v>190</v>
+        <v>42</v>
       </c>
       <c r="Y15" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="Z15" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="AC15" t="s">
         <v>80</v>
@@ -2134,22 +2070,25 @@
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C16" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="D16" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="E16" t="s">
         <v>75</v>
       </c>
       <c r="F16" t="s">
-        <v>140</v>
+        <v>122</v>
+      </c>
+      <c r="G16" t="s">
+        <v>78</v>
       </c>
       <c r="I16" t="s">
         <v>76</v>
@@ -2179,25 +2118,25 @@
         <v>79</v>
       </c>
       <c r="T16">
+        <v>7</v>
+      </c>
+      <c r="U16">
+        <v>9</v>
+      </c>
+      <c r="V16">
         <v>8</v>
       </c>
-      <c r="U16">
+      <c r="W16">
         <v>4</v>
       </c>
-      <c r="V16">
-        <v>4</v>
-      </c>
-      <c r="W16">
-        <v>5</v>
-      </c>
       <c r="X16">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="Y16" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="Z16" t="s">
-        <v>142</v>
+        <v>107</v>
       </c>
       <c r="AC16" t="s">
         <v>80</v>
@@ -2208,25 +2147,22 @@
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C17" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="D17" t="s">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="F17" t="s">
-        <v>144</v>
-      </c>
-      <c r="G17" t="s">
-        <v>78</v>
+        <v>125</v>
       </c>
       <c r="I17" t="s">
         <v>76</v>
@@ -2256,25 +2192,25 @@
         <v>79</v>
       </c>
       <c r="T17">
+        <v>2</v>
+      </c>
+      <c r="U17">
         <v>3</v>
       </c>
-      <c r="U17">
-        <v>8</v>
-      </c>
       <c r="V17">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W17">
         <v>7</v>
       </c>
       <c r="X17">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="Y17" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="Z17" t="s">
-        <v>146</v>
+        <v>111</v>
       </c>
       <c r="AC17" t="s">
         <v>80</v>
@@ -2285,22 +2221,22 @@
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>148</v>
+        <v>127</v>
       </c>
       <c r="D18" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="E18" t="s">
         <v>75</v>
       </c>
       <c r="F18" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="I18" t="s">
         <v>76</v>
@@ -2330,25 +2266,25 @@
         <v>79</v>
       </c>
       <c r="T18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V18">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="W18">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="X18">
-        <v>210</v>
+        <v>84</v>
       </c>
       <c r="Y18" t="s">
-        <v>148</v>
+        <v>127</v>
       </c>
       <c r="Z18" t="s">
-        <v>149</v>
+        <v>112</v>
       </c>
       <c r="AC18" t="s">
         <v>80</v>
@@ -2359,25 +2295,22 @@
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="D19" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="E19" t="s">
-        <v>153</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
-        <v>151</v>
-      </c>
-      <c r="G19" t="s">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="I19" t="s">
         <v>76</v>
@@ -2407,25 +2340,25 @@
         <v>79</v>
       </c>
       <c r="T19">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="U19">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="V19">
         <v>8</v>
       </c>
       <c r="W19">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="X19">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="Y19" t="s">
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="Z19" t="s">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="AC19" t="s">
         <v>80</v>
@@ -2436,22 +2369,25 @@
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>131</v>
       </c>
       <c r="B20" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>132</v>
       </c>
       <c r="D20" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
       <c r="E20" t="s">
         <v>75</v>
       </c>
       <c r="F20" t="s">
-        <v>85</v>
+        <v>132</v>
+      </c>
+      <c r="G20" t="s">
+        <v>78</v>
       </c>
       <c r="I20" t="s">
         <v>76</v>
@@ -2481,25 +2417,25 @@
         <v>79</v>
       </c>
       <c r="T20">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V20">
         <v>5</v>
       </c>
       <c r="W20">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="X20">
-        <v>135</v>
+        <v>27</v>
       </c>
       <c r="Y20" t="s">
-        <v>85</v>
+        <v>132</v>
       </c>
       <c r="Z20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AC20" t="s">
         <v>80</v>
@@ -2510,22 +2446,22 @@
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="B21" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="D21" t="s">
-        <v>158</v>
+        <v>118</v>
       </c>
       <c r="E21" t="s">
         <v>75</v>
       </c>
       <c r="F21" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="I21" t="s">
         <v>76</v>
@@ -2555,25 +2491,25 @@
         <v>79</v>
       </c>
       <c r="T21">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U21">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="V21">
         <v>6</v>
       </c>
       <c r="W21">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X21">
-        <v>117</v>
+        <v>144</v>
       </c>
       <c r="Y21" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="Z21" t="s">
-        <v>159</v>
+        <v>88</v>
       </c>
       <c r="AC21" t="s">
         <v>80</v>
@@ -2584,25 +2520,22 @@
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="B22" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="C22" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="D22" t="s">
-        <v>158</v>
+        <v>123</v>
       </c>
       <c r="E22" t="s">
         <v>75</v>
       </c>
       <c r="F22" t="s">
-        <v>161</v>
-      </c>
-      <c r="G22" t="s">
-        <v>78</v>
+        <v>137</v>
       </c>
       <c r="I22" t="s">
         <v>76</v>
@@ -2632,25 +2565,25 @@
         <v>79</v>
       </c>
       <c r="T22">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U22">
+        <v>1</v>
+      </c>
+      <c r="V22">
         <v>4</v>
-      </c>
-      <c r="V22">
-        <v>7</v>
       </c>
       <c r="W22">
         <v>6</v>
       </c>
       <c r="X22">
-        <v>108</v>
+        <v>42</v>
       </c>
       <c r="Y22" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="Z22" t="s">
-        <v>162</v>
+        <v>89</v>
       </c>
       <c r="AC22" t="s">
         <v>80</v>
@@ -2661,25 +2594,22 @@
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>163</v>
+        <v>138</v>
       </c>
       <c r="B23" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
-        <v>164</v>
+        <v>139</v>
       </c>
       <c r="D23" t="s">
-        <v>165</v>
+        <v>123</v>
       </c>
       <c r="E23" t="s">
         <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>164</v>
-      </c>
-      <c r="G23" t="s">
-        <v>78</v>
+        <v>139</v>
       </c>
       <c r="I23" t="s">
         <v>76</v>
@@ -2709,25 +2639,25 @@
         <v>79</v>
       </c>
       <c r="T23">
+        <v>5</v>
+      </c>
+      <c r="U23">
+        <v>6</v>
+      </c>
+      <c r="V23">
         <v>9</v>
       </c>
-      <c r="U23">
-        <v>8</v>
-      </c>
-      <c r="V23">
-        <v>4</v>
-      </c>
       <c r="W23">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="X23">
-        <v>21</v>
+        <v>180</v>
       </c>
       <c r="Y23" t="s">
-        <v>164</v>
+        <v>139</v>
       </c>
       <c r="Z23" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="AC23" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
feat: Enhance training output handling with village and amount fields
- Added 'village' and 'amount' fields to the TrainingOutputHandler.
- Updated validation logic to ensure 'amount' is required, numeric, and greater than zero.
- Implemented a method to retrieve the first available dropdown option for 'village'.
- Modified the Excel reader to map 'village' and 'amount' columns correctly.
- Updated migration scripts to include new headers for 'village' and 'amount'.
- Added unit tests to validate the new fields and their integration with Excel input.
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Automation\egram_bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D7A009-1574-4826-BDC8-7CEC3E5069FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49852B07-56D2-4E55-BFCB-48387AE71900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activities" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <sheet name="Beneficiaries" sheetId="5" r:id="rId5"/>
     <sheet name="Asset" sheetId="6" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Activities!$A$1:$AG$1</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="166">
   <si>
     <t>Activity_Key</t>
   </si>
@@ -48,6 +45,9 @@
     <t>activity_description</t>
   </si>
   <si>
+    <t>vprp_plan</t>
+  </si>
+  <si>
     <t>pdi_indicator</t>
   </si>
   <si>
@@ -126,9 +126,276 @@
     <t>error_message</t>
   </si>
   <si>
+    <t>ACT-0063</t>
+  </si>
+  <si>
+    <t>Theme 3 - Child Friendly Village</t>
+  </si>
+  <si>
+    <t>Awareness Campaign on services of ICDS: Child rights &amp; protection</t>
+  </si>
+  <si>
+    <t>Women and child development</t>
+  </si>
+  <si>
+    <t>Community Works</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>New/Fresh</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>Mahatma Gandhi National Rural Employment Guarantee Scheme (MGNREGS) - Center Scheme</t>
+  </si>
+  <si>
+    <t>Training/Capacity Building</t>
+  </si>
+  <si>
+    <t>Save and Forward</t>
+  </si>
+  <si>
+    <t>ACT-0064</t>
+  </si>
+  <si>
+    <t>Awareness Program/ Rallies / Street Play on child marriage, child labour, child marriage, trafficking</t>
+  </si>
+  <si>
+    <t>Social welfare</t>
+  </si>
+  <si>
+    <t>Deendayal Upadhyaya Grameen Kaushalya Yojana(DDUGKY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0065</t>
+  </si>
+  <si>
+    <t>Awareness Program/ Rallies/ Campaign on importance of education/ vocational / technical education</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>National Social Assistance Programme (NSAP) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0066</t>
+  </si>
+  <si>
+    <t>Awareness Program/Campaign - Health, Nutrion &amp; Hygiene  practices</t>
+  </si>
+  <si>
+    <t>Awareness Program/Campaign - Health, Nutrion &amp; Hygiene practices</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri AwasYojana Gramin PMAY (G) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0067</t>
+  </si>
+  <si>
+    <t>Awareness camp on different schemes related to special children</t>
+  </si>
+  <si>
+    <t>Swachh Bharat Mission (Gramin) (SBM (G)] - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0068</t>
+  </si>
+  <si>
+    <t>Awareness on gender discrimination and gender equality</t>
+  </si>
+  <si>
+    <t>Jal Jeevan Mission (JJM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0069</t>
+  </si>
+  <si>
+    <t>Capacity Building &amp; Training of Children</t>
+  </si>
+  <si>
+    <t>Deendayal Upadhyaya Gram Jyoti Yojana (DDUGJY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0070</t>
+  </si>
+  <si>
+    <t>Child Participation, Leadership Strengthening &amp; Facilitation</t>
+  </si>
+  <si>
+    <t>Whether the activity is for Elementary/Primary Education</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0081</t>
+  </si>
+  <si>
+    <t>Institutional Strengthening &amp; Convergence on child related issues</t>
+  </si>
+  <si>
+    <t>National Health Mission (NHM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0087</t>
+  </si>
+  <si>
+    <t>Providing Educational Materials /Special Coaching Support to the student</t>
+  </si>
+  <si>
+    <t>Mid-Day Meal Scheme (MDM) - Center Scheme</t>
+  </si>
+  <si>
     <t>ACT-0001</t>
   </si>
   <si>
+    <t>Theme 1 - Poverty Free and Enhanced Livelihoods Village</t>
+  </si>
+  <si>
+    <t>Conduct IEC/awareness and  inclusion camps for social protection and beneficiary-oriented schemes</t>
+  </si>
+  <si>
+    <t>Conduct IEC/awareness and inclusion camps for social protection and beneficiary-oriented schemes</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Matru Vandana Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0002</t>
+  </si>
+  <si>
+    <t>Create awareness on FPOs and support formation/strngthening of FPOs through farmer mobilisation</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
+    <t>Pradhan Mantri Ujjwala Yojana - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0003</t>
+  </si>
+  <si>
+    <t>Create awareness on volunteering and community support initiatices, including animal welfare activities</t>
+  </si>
+  <si>
+    <t>Animal husbandry</t>
+  </si>
+  <si>
+    <t>Antodaya Anna Yojana - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0015</t>
+  </si>
+  <si>
+    <t>Facilitate formation oh SHGs and provide support for strengthening SHGs in Gram Panchayats</t>
+  </si>
+  <si>
+    <t>Poverty allevation programme</t>
+  </si>
+  <si>
+    <t>Samagara Shikha Abhiyan - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0020</t>
+  </si>
+  <si>
+    <t>Facilitation/provision of skill development training</t>
+  </si>
+  <si>
+    <t>Technical training and vocational education</t>
+  </si>
+  <si>
+    <t>Beneficiary Oriented Programmes</t>
+  </si>
+  <si>
+    <t>Poshan Abhiyan/ICDS - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0028</t>
+  </si>
+  <si>
+    <t>Organise career counselling camps to promote self-employment opportunities at the GP level</t>
+  </si>
+  <si>
+    <t>Beti Bachao Beti Padao - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0036</t>
+  </si>
+  <si>
+    <t>Theme 2 - Healthy Village</t>
+  </si>
+  <si>
+    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of Vector Borne Diseases (VBD)</t>
+  </si>
+  <si>
+    <t>Health</t>
+  </si>
+  <si>
+    <t>National Rural Livelihood Mission (NRLM) - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0037</t>
+  </si>
+  <si>
+    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of anaemia; vicious cycle of anaemia</t>
+  </si>
+  <si>
+    <t>Pashudhan Scheme - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0043</t>
+  </si>
+  <si>
+    <t>Oraginizing awareness camp/ program on significance of health &amp; nutrition</t>
+  </si>
+  <si>
+    <t>Family welfare</t>
+  </si>
+  <si>
+    <t>Matsaya Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0044</t>
+  </si>
+  <si>
+    <t>Oranizing Training of Mid Wives on safe &amp; institutional delivery</t>
+  </si>
+  <si>
+    <t>Janani Surakha Yojna - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0046</t>
+  </si>
+  <si>
+    <t>Organize Mental Health Awareness Camps  &amp; Development of IEC materials on Mental Health</t>
+  </si>
+  <si>
+    <t>Organize Mental Health Awareness Camps &amp; Development of IEC materials on Mental Health</t>
+  </si>
+  <si>
+    <t>Ayushman Bharat - Center Scheme</t>
+  </si>
+  <si>
+    <t>ACT-0047</t>
+  </si>
+  <si>
+    <t>Organizing Awareness &amp; IEC campaign on Health Schemes/ Program</t>
+  </si>
+  <si>
+    <t>National Biogas and Manure Management Programme - Center Scheme</t>
+  </si>
+  <si>
     <t>Field</t>
   </si>
   <si>
@@ -237,6 +504,12 @@
     <t>Subject of Training</t>
   </si>
   <si>
+    <t>Village</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
     <t>Total Trainees</t>
   </si>
   <si>
@@ -250,270 +523,6 @@
   </si>
   <si>
     <t>50</t>
-  </si>
-  <si>
-    <t>vprp_plan</t>
-  </si>
-  <si>
-    <t>Community Works</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>New/Fresh</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>April</t>
-  </si>
-  <si>
-    <t>Training/Capacity Building</t>
-  </si>
-  <si>
-    <t>Save and Forward</t>
-  </si>
-  <si>
-    <t>Social welfare</t>
-  </si>
-  <si>
-    <t>National Social Assistance Programme (NSAP) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Theme 1 - Poverty Free and Enhanced Livelihoods Village</t>
-  </si>
-  <si>
-    <t>Conduct IEC/awareness and inclusion camps for social protection and beneficiary-oriented schemes</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Ujjwala Yojana - Center Scheme</t>
-  </si>
-  <si>
-    <t>Matsaya Yojna - Center Scheme</t>
-  </si>
-  <si>
-    <t>Janani Surakha Yojna - Center Scheme</t>
-  </si>
-  <si>
-    <t>Ayushman Bharat - Center Scheme</t>
-  </si>
-  <si>
-    <t>National Biogas and Manure Management Programme - Center Scheme</t>
-  </si>
-  <si>
-    <t>Conduct IEC/awareness and  inclusion camps for social protection and beneficiary-oriented schemes</t>
-  </si>
-  <si>
-    <t>Mahatma Gandhi National Rural Employment Guarantee Scheme (MGNREGS) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Deendayal Upadhyaya Grameen Kaushalya Yojana(DDUGKY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri AwasYojana Gramin PMAY (G) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Swachh Bharat Mission (Gramin) (SBM (G)] - Center Scheme</t>
-  </si>
-  <si>
-    <t>Jal Jeevan Mission (JJM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Deendayal Upadhyaya Gram Jyoti Yojana (DDUGJY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
-  </si>
-  <si>
-    <t>National Health Mission (NHM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Mid-Day Meal Scheme (MDM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Pradhan Mantri Matru Vandana Yojna - Center Scheme</t>
-  </si>
-  <si>
-    <t>Antodaya Anna Yojana - Center Scheme</t>
-  </si>
-  <si>
-    <t>Samagara Shikha Abhiyan - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0002</t>
-  </si>
-  <si>
-    <t>Create awareness on FPOs and support formation/strngthening of FPOs through farmer mobilisation</t>
-  </si>
-  <si>
-    <t>Agriculture</t>
-  </si>
-  <si>
-    <t>Poshan Abhiyan/ICDS - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0003</t>
-  </si>
-  <si>
-    <t>Create awareness on volunteering and community support initiatices, including animal welfare activities</t>
-  </si>
-  <si>
-    <t>Animal husbandry</t>
-  </si>
-  <si>
-    <t>Beti Bachao Beti Padao - Center Scheme</t>
-  </si>
-  <si>
-    <t>National Rural Livelihood Mission (NRLM) - Center Scheme</t>
-  </si>
-  <si>
-    <t>Beneficiary Oriented Programmes</t>
-  </si>
-  <si>
-    <t>Pashudhan Scheme - Center Scheme</t>
-  </si>
-  <si>
-    <t>ACT-0036</t>
-  </si>
-  <si>
-    <t>Theme 2 - Healthy Village</t>
-  </si>
-  <si>
-    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of Vector Borne Diseases (VBD)</t>
-  </si>
-  <si>
-    <t>Health</t>
-  </si>
-  <si>
-    <t>ACT-0037</t>
-  </si>
-  <si>
-    <t>Organizing awareness Progarm &amp; IEC campaign on symptoms of anaemia; vicious cycle of anaemia</t>
-  </si>
-  <si>
-    <t>ACT-0043</t>
-  </si>
-  <si>
-    <t>Oraginizing awareness camp/ program on significance of health &amp; nutrition</t>
-  </si>
-  <si>
-    <t>Family welfare</t>
-  </si>
-  <si>
-    <t>ACT-0044</t>
-  </si>
-  <si>
-    <t>Oranizing Training of Mid Wives on safe &amp; institutional delivery</t>
-  </si>
-  <si>
-    <t>ACT-0046</t>
-  </si>
-  <si>
-    <t>Organize Mental Health Awareness Camps  &amp; Development of IEC materials on Mental Health</t>
-  </si>
-  <si>
-    <t>Organize Mental Health Awareness Camps &amp; Development of IEC materials on Mental Health</t>
-  </si>
-  <si>
-    <t>ACT-0047</t>
-  </si>
-  <si>
-    <t>Organizing Awareness &amp; IEC campaign on Health Schemes/ Program</t>
-  </si>
-  <si>
-    <t>ACT-0048</t>
-  </si>
-  <si>
-    <t>Organizing Awareness Campaign/ Program including Nukkad Natak/Street Play on Maternal and Child health</t>
-  </si>
-  <si>
-    <t>Cultural activities</t>
-  </si>
-  <si>
-    <t>ACT-0051</t>
-  </si>
-  <si>
-    <t>Organizing awareness camp about child heath through campaign</t>
-  </si>
-  <si>
-    <t>ACT-0052</t>
-  </si>
-  <si>
-    <t>Organizing awareness camp on institutional delivery and early registration to the hospitals for ante-natal chaeck up &amp; post natal check up of pregnanat mothers</t>
-  </si>
-  <si>
-    <t>ACT-0053</t>
-  </si>
-  <si>
-    <t>Organizing awareness camp on rountine immunization of children</t>
-  </si>
-  <si>
-    <t>ACT-0015</t>
-  </si>
-  <si>
-    <t>Facilitate formation oh SHGs and provide support for strengthening SHGs in Gram Panchayats</t>
-  </si>
-  <si>
-    <t>Poverty allevation programme</t>
-  </si>
-  <si>
-    <t>ACT-0020</t>
-  </si>
-  <si>
-    <t>Facilitation/provision of skill development training</t>
-  </si>
-  <si>
-    <t>Technical training and vocational education</t>
-  </si>
-  <si>
-    <t>ACT-0028</t>
-  </si>
-  <si>
-    <t>Organise career counselling camps to promote self-employment opportunities at the GP level</t>
-  </si>
-  <si>
-    <t>ACT-0306</t>
-  </si>
-  <si>
-    <t>Theme 8 - Village with Good Governance</t>
-  </si>
-  <si>
-    <t>Capacity Building &amp; Training of Elected Representatives, Functionaries &amp; other stakeholders</t>
-  </si>
-  <si>
-    <t>ACT-0310</t>
-  </si>
-  <si>
-    <t>Cost for Disaster Readiness, relief and mitigation activities (Training, planning, survey etc)</t>
-  </si>
-  <si>
-    <t>Adult and non-formal education</t>
-  </si>
-  <si>
-    <t>ACT-0313</t>
-  </si>
-  <si>
-    <t>IEC &amp; Awareness Campaign for active participation in Gram Sabha, Ward Sabha, Mahila Sabha</t>
-  </si>
-  <si>
-    <t>ACT-0314</t>
-  </si>
-  <si>
-    <t>IEC &amp; Awareness campaign on SHG-PRI Convergence /Public Services/ Service Delivery Provisions/ RTI/Grivences</t>
-  </si>
-  <si>
-    <t>ACT-0315</t>
-  </si>
-  <si>
-    <t>IEC &amp; Awareness on disaster preparedness and mitigation</t>
-  </si>
-  <si>
-    <t>ACT-0317</t>
-  </si>
-  <si>
-    <t>Organising of Gram Sabha/ Ward Sabha/ Mahila Sabha/ GPDP</t>
   </si>
 </sst>
 </file>
@@ -889,7 +898,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" customWidth="1"/>
     <col min="3" max="3" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -942,117 +951,117 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AA1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AD1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="AE1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="AF1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AG1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J2" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K2" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N2" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O2">
         <v>1</v>
@@ -1067,66 +1076,69 @@
         <v>2026</v>
       </c>
       <c r="S2" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T2">
         <v>8</v>
       </c>
       <c r="U2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W2">
         <v>9</v>
       </c>
       <c r="X2">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="Y2" t="s">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="Z2" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="AC2" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD2" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>152</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>153</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>152</v>
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>40</v>
       </c>
       <c r="I3" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J3" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K3" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N3" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O3">
         <v>1</v>
@@ -1141,66 +1153,69 @@
         <v>2026</v>
       </c>
       <c r="S3" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="V3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="X3">
-        <v>198</v>
+        <v>72</v>
       </c>
       <c r="Y3" t="s">
-        <v>152</v>
+        <v>46</v>
       </c>
       <c r="Z3" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="AC3" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD3" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>155</v>
+        <v>50</v>
+      </c>
+      <c r="G4" t="s">
+        <v>40</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J4" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K4" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N4" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O4">
         <v>1</v>
@@ -1215,66 +1230,66 @@
         <v>2026</v>
       </c>
       <c r="S4" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T4">
+        <v>4</v>
+      </c>
+      <c r="U4">
+        <v>4</v>
+      </c>
+      <c r="V4">
+        <v>5</v>
+      </c>
+      <c r="W4">
         <v>3</v>
       </c>
-      <c r="U4">
-        <v>5</v>
-      </c>
-      <c r="V4">
-        <v>3</v>
-      </c>
-      <c r="W4">
-        <v>1</v>
-      </c>
       <c r="X4">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="Y4" t="s">
-        <v>155</v>
+        <v>50</v>
       </c>
       <c r="Z4" t="s">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="AC4" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD4" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
       <c r="D5" t="s">
-        <v>153</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>157</v>
+        <v>55</v>
       </c>
       <c r="I5" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J5" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N5" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O5">
         <v>1</v>
@@ -1289,66 +1304,66 @@
         <v>2026</v>
       </c>
       <c r="S5" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U5">
         <v>8</v>
       </c>
       <c r="V5">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="W5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X5">
-        <v>34</v>
+        <v>138</v>
       </c>
       <c r="Y5" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
       <c r="Z5" t="s">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="AC5" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD5" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>158</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>159</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>153</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>159</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J6" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K6" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N6" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O6">
         <v>1</v>
@@ -1363,66 +1378,66 @@
         <v>2026</v>
       </c>
       <c r="S6" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T6">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="U6">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="V6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="X6">
-        <v>160</v>
+        <v>132</v>
       </c>
       <c r="Y6" t="s">
-        <v>159</v>
+        <v>58</v>
       </c>
       <c r="Z6" t="s">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="AC6" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD6" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>160</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>161</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>82</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
-        <v>161</v>
+        <v>61</v>
       </c>
       <c r="I7" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J7" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K7" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N7" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O7">
         <v>1</v>
@@ -1437,66 +1452,66 @@
         <v>2026</v>
       </c>
       <c r="S7" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T7">
+        <v>10</v>
+      </c>
+      <c r="U7">
+        <v>5</v>
+      </c>
+      <c r="V7">
         <v>8</v>
       </c>
-      <c r="U7">
-        <v>8</v>
-      </c>
-      <c r="V7">
-        <v>10</v>
-      </c>
       <c r="W7">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="X7">
-        <v>26</v>
+        <v>161</v>
       </c>
       <c r="Y7" t="s">
-        <v>161</v>
+        <v>61</v>
       </c>
       <c r="Z7" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="AC7" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD7" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J8" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K8" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N8" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O8">
         <v>1</v>
@@ -1511,66 +1526,69 @@
         <v>2026</v>
       </c>
       <c r="S8" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T8">
+        <v>3</v>
+      </c>
+      <c r="U8">
+        <v>9</v>
+      </c>
+      <c r="V8">
         <v>7</v>
       </c>
-      <c r="U8">
+      <c r="W8">
         <v>8</v>
       </c>
-      <c r="V8">
-        <v>8</v>
-      </c>
-      <c r="W8">
-        <v>10</v>
-      </c>
       <c r="X8">
-        <v>230</v>
+        <v>152</v>
       </c>
       <c r="Y8" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="Z8" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="AC8" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD8" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J9" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K9" t="s">
-        <v>77</v>
+        <v>39</v>
+      </c>
+      <c r="M9" t="s">
+        <v>68</v>
       </c>
       <c r="N9" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O9">
         <v>1</v>
@@ -1585,69 +1603,69 @@
         <v>2026</v>
       </c>
       <c r="S9" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T9">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V9">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W9">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="X9">
-        <v>230</v>
+        <v>27</v>
       </c>
       <c r="Y9" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="Z9" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="AC9" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD9" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F10" t="s">
-        <v>109</v>
-      </c>
-      <c r="G10" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="I10" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J10" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K10" t="s">
-        <v>77</v>
+        <v>39</v>
+      </c>
+      <c r="M10" t="s">
+        <v>68</v>
       </c>
       <c r="N10" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O10">
         <v>1</v>
@@ -1662,66 +1680,66 @@
         <v>2026</v>
       </c>
       <c r="S10" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W10">
         <v>5</v>
       </c>
       <c r="X10">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="Y10" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
       <c r="Z10" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="AC10" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD10" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>141</v>
+        <v>74</v>
       </c>
       <c r="D11" t="s">
-        <v>142</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>141</v>
+        <v>74</v>
       </c>
       <c r="I11" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J11" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K11" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N11" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -1736,69 +1754,66 @@
         <v>2026</v>
       </c>
       <c r="S11" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U11">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="V11">
         <v>2</v>
       </c>
       <c r="W11">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="X11">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="Y11" t="s">
-        <v>141</v>
+        <v>74</v>
       </c>
       <c r="Z11" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AC11" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD11" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>144</v>
+        <v>78</v>
       </c>
       <c r="D12" t="s">
-        <v>145</v>
+        <v>47</v>
       </c>
       <c r="E12" t="s">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
-        <v>144</v>
-      </c>
-      <c r="G12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I12" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J12" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K12" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N12" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O12">
         <v>1</v>
@@ -1813,66 +1828,66 @@
         <v>2026</v>
       </c>
       <c r="S12" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T12">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U12">
         <v>9</v>
       </c>
       <c r="V12">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="W12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X12">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="Y12" t="s">
-        <v>144</v>
+        <v>78</v>
       </c>
       <c r="Z12" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="AC12" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD12" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>146</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>147</v>
+        <v>82</v>
       </c>
       <c r="D13" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>82</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J13" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K13" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N13" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O13">
         <v>1</v>
@@ -1887,66 +1902,69 @@
         <v>2026</v>
       </c>
       <c r="S13" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T13">
+        <v>8</v>
+      </c>
+      <c r="U13">
+        <v>3</v>
+      </c>
+      <c r="V13">
         <v>6</v>
       </c>
-      <c r="U13">
-        <v>2</v>
-      </c>
-      <c r="V13">
-        <v>7</v>
-      </c>
       <c r="W13">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="X13">
-        <v>150</v>
+        <v>102</v>
       </c>
       <c r="Y13" t="s">
-        <v>147</v>
+        <v>82</v>
       </c>
       <c r="Z13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AC13" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD13" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>117</v>
+        <v>86</v>
       </c>
       <c r="D14" t="s">
-        <v>118</v>
+        <v>87</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
-        <v>117</v>
+        <v>86</v>
+      </c>
+      <c r="G14" t="s">
+        <v>40</v>
       </c>
       <c r="I14" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J14" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K14" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N14" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O14">
         <v>1</v>
@@ -1961,69 +1979,66 @@
         <v>2026</v>
       </c>
       <c r="S14" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T14">
         <v>3</v>
       </c>
       <c r="U14">
+        <v>4</v>
+      </c>
+      <c r="V14">
         <v>9</v>
       </c>
-      <c r="V14">
-        <v>10</v>
-      </c>
       <c r="W14">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="X14">
-        <v>176</v>
+        <v>48</v>
       </c>
       <c r="Y14" t="s">
-        <v>117</v>
+        <v>86</v>
       </c>
       <c r="Z14" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="AC14" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD14" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>120</v>
-      </c>
-      <c r="G15" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="I15" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J15" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K15" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N15" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O15">
         <v>1</v>
@@ -2038,69 +2053,69 @@
         <v>2026</v>
       </c>
       <c r="S15" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T15">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="V15">
+        <v>5</v>
+      </c>
+      <c r="W15">
         <v>4</v>
       </c>
-      <c r="W15">
-        <v>2</v>
-      </c>
       <c r="X15">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="Y15" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="Z15" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="AC15" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD15" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="D16" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="F16" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="G16" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="I16" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J16" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K16" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N16" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O16">
         <v>1</v>
@@ -2115,66 +2130,66 @@
         <v>2026</v>
       </c>
       <c r="S16" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U16">
+        <v>8</v>
+      </c>
+      <c r="V16">
         <v>9</v>
       </c>
-      <c r="V16">
-        <v>8</v>
-      </c>
       <c r="W16">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="X16">
-        <v>96</v>
+        <v>207</v>
       </c>
       <c r="Y16" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="Z16" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="AC16" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD16" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="F17" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="I17" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J17" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K17" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N17" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O17">
         <v>1</v>
@@ -2189,66 +2204,66 @@
         <v>2026</v>
       </c>
       <c r="S17" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T17">
+        <v>9</v>
+      </c>
+      <c r="U17">
         <v>2</v>
       </c>
-      <c r="U17">
-        <v>3</v>
-      </c>
       <c r="V17">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="W17">
         <v>7</v>
       </c>
       <c r="X17">
-        <v>77</v>
+        <v>140</v>
       </c>
       <c r="Y17" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="Z17" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="AC17" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD17" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C18" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
       <c r="D18" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F18" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="I18" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J18" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K18" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N18" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O18">
         <v>1</v>
@@ -2263,66 +2278,69 @@
         <v>2026</v>
       </c>
       <c r="S18" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T18">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="U18">
+        <v>7</v>
+      </c>
+      <c r="V18">
         <v>3</v>
       </c>
-      <c r="V18">
-        <v>10</v>
-      </c>
       <c r="W18">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X18">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="Y18" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
       <c r="Z18" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="AC18" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD18" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="B19" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>130</v>
+        <v>107</v>
       </c>
       <c r="D19" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F19" t="s">
-        <v>130</v>
+        <v>107</v>
+      </c>
+      <c r="G19" t="s">
+        <v>40</v>
       </c>
       <c r="I19" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J19" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K19" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N19" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -2337,69 +2355,69 @@
         <v>2026</v>
       </c>
       <c r="S19" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T19">
+        <v>9</v>
+      </c>
+      <c r="U19">
+        <v>1</v>
+      </c>
+      <c r="V19">
         <v>10</v>
       </c>
-      <c r="U19">
-        <v>10</v>
-      </c>
-      <c r="V19">
-        <v>8</v>
-      </c>
       <c r="W19">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X19">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="Y19" t="s">
-        <v>130</v>
+        <v>107</v>
       </c>
       <c r="Z19" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="AC19" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD19" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="D20" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F20" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="G20" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="I20" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J20" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K20" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N20" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O20">
         <v>1</v>
@@ -2414,66 +2432,66 @@
         <v>2026</v>
       </c>
       <c r="S20" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U20">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="V20">
         <v>5</v>
       </c>
       <c r="W20">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="X20">
-        <v>27</v>
+        <v>153</v>
       </c>
       <c r="Y20" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="Z20" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AC20" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD20" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="D21" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="E21" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="F21" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="I21" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J21" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K21" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N21" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O21">
         <v>1</v>
@@ -2488,66 +2506,66 @@
         <v>2026</v>
       </c>
       <c r="S21" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T21">
+        <v>8</v>
+      </c>
+      <c r="U21">
         <v>4</v>
       </c>
-      <c r="U21">
+      <c r="V21">
         <v>8</v>
       </c>
-      <c r="V21">
-        <v>6</v>
-      </c>
       <c r="W21">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="X21">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="Y21" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="Z21" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="AC21" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD21" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="B22" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F22" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="I22" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J22" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K22" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N22" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O22">
         <v>1</v>
@@ -2562,66 +2580,66 @@
         <v>2026</v>
       </c>
       <c r="S22" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U22">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="V22">
         <v>4</v>
       </c>
       <c r="W22">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="X22">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="Y22" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="Z22" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="AC22" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD22" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C23" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E23" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="F23" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="I23" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J23" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="K23" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="N23" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O23">
         <v>1</v>
@@ -2636,39 +2654,39 @@
         <v>2026</v>
       </c>
       <c r="S23" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="T23">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U23">
+        <v>9</v>
+      </c>
+      <c r="V23">
+        <v>8</v>
+      </c>
+      <c r="W23">
         <v>6</v>
       </c>
-      <c r="V23">
-        <v>9</v>
-      </c>
-      <c r="W23">
-        <v>9</v>
-      </c>
       <c r="X23">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="Y23" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="Z23" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="AC23" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AD23" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -2683,10 +2701,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -2694,7 +2712,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>35</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2702,7 +2720,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>36</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -2710,7 +2728,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2718,7 +2736,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>38</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2726,135 +2744,135 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>39</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>40</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>41</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>42</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>43</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>44</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>45</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>47</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>48</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>49</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>50</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>51</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>52</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>52</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>52</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>53</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2863,50 +2881,50 @@
     </row>
     <row r="24" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>54</v>
+        <v>144</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>55</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>56</v>
+        <v>146</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>57</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>58</v>
+        <v>148</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>59</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>61</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>62</v>
+        <v>152</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>63</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>64</v>
+        <v>154</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>65</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2916,7 +2934,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -2926,44 +2944,53 @@
     <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>157</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>158</v>
       </c>
       <c r="E1" t="s">
-        <v>69</v>
+        <v>159</v>
       </c>
       <c r="F1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+      <c r="G1" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F2" t="s">
-        <v>73</v>
+        <v>164</v>
+      </c>
+      <c r="F2">
+        <v>10000</v>
+      </c>
+      <c r="G2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H2" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>